<commit_message>
Initial commit: currency tracker ЦБ РФ
</commit_message>
<xml_diff>
--- a/history.xlsx
+++ b/history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -492,6 +492,22 @@
         <v>10.9536</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>05.06.2026 07:18</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>74.29559999999999</v>
+      </c>
+      <c r="C5" t="n">
+        <v>86.27119999999999</v>
+      </c>
+      <c r="D5" t="n">
+        <v>10.9536</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>